<commit_message>
Admin: edit data/team.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/team.xlsx
+++ b/data/team.xlsx
@@ -620,7 +620,7 @@
         <v>Creative and Marketing Team</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>assets/images/team/deepika-harkande.jpg</v>
       </c>
     </row>
     <row r="17">
@@ -628,7 +628,7 @@
         <v>Divya Chaudhari</v>
       </c>
       <c r="B17" t="str">
-        <v>Social Media Head</v>
+        <v>Social Media Lead</v>
       </c>
       <c r="C17" t="str">
         <v>Creative and Marketing Team</v>

</xml_diff>